<commit_message>
Update Pendapatan per Kapita Pesisir
</commit_message>
<xml_diff>
--- a/LDM.xlsx
+++ b/LDM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\1_LASSO\LAS_Simulation_Jateng\I-O_Analysis\Regional-Economy---Jawa-Tengah\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://icrafcifor-my.sharepoint.com/personal/d_bodro_landscapealliance_org/Documents/Documents/GitHub/Regional-Economy---Jawa-Tengah/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B687B574-154E-4477-83B2-608DCE44F8A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{B687B574-154E-4477-83B2-608DCE44F8A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{712F2B52-FF42-4C2C-83FC-31FCDBF28E3D}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{353B98BA-F33D-49CB-8D7C-42B1DBC60FEF}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{353B98BA-F33D-49CB-8D7C-42B1DBC60FEF}"/>
   </bookViews>
   <sheets>
     <sheet name="LDM" sheetId="1" r:id="rId1"/>
@@ -36,10 +36,6 @@
     </ext>
   </extLst>
 </workbook>
-</file>
-
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -241,87 +237,87 @@
   <sheetPr>
     <tabColor theme="3" tint="0.499984740745262"/>
   </sheetPr>
-  <dimension ref="A1:Z66"/>
-  <sheetFormatPr defaultRowHeight="14"/>
+  <dimension ref="A1:Z67"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <sheetData>
     <row r="1" spans="1:26">
       <c r="A1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C1">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D1">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E1">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F1">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G1">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="H1">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="I1">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="J1">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K1">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="L1">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="M1">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="N1">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="O1">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="P1">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="Q1">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="R1">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="S1">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="T1">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="U1">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="V1">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="W1">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="X1">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="Y1">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="Z1">
-        <v>0</v>
+        <v>26</v>
       </c>
     </row>
     <row r="2" spans="1:26">
@@ -377,10 +373,10 @@
         <v>0</v>
       </c>
       <c r="R2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S2">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="T2">
         <v>0</v>
@@ -439,7 +435,7 @@
         <v>0</v>
       </c>
       <c r="L3">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="M3">
         <v>0</v>
@@ -519,10 +515,10 @@
         <v>0</v>
       </c>
       <c r="L4">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="M4">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="N4">
         <v>0</v>
@@ -602,7 +598,7 @@
         <v>0</v>
       </c>
       <c r="M5">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="N5">
         <v>0</v>
@@ -676,7 +672,7 @@
         <v>0</v>
       </c>
       <c r="K6">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="L6">
         <v>0</v>
@@ -753,34 +749,34 @@
         <v>0</v>
       </c>
       <c r="J7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K7">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
       <c r="L7">
+        <v>0</v>
+      </c>
+      <c r="M7">
+        <v>0</v>
+      </c>
+      <c r="N7">
+        <v>0</v>
+      </c>
+      <c r="O7">
+        <v>0</v>
+      </c>
+      <c r="P7">
+        <v>0</v>
+      </c>
+      <c r="Q7">
+        <v>0</v>
+      </c>
+      <c r="R7">
+        <v>0</v>
+      </c>
+      <c r="S7">
         <v>0.2</v>
-      </c>
-      <c r="M7">
-        <v>0</v>
-      </c>
-      <c r="N7">
-        <v>0.1</v>
-      </c>
-      <c r="O7">
-        <v>0.1</v>
-      </c>
-      <c r="P7">
-        <v>0</v>
-      </c>
-      <c r="Q7">
-        <v>0</v>
-      </c>
-      <c r="R7">
-        <v>0</v>
-      </c>
-      <c r="S7">
-        <v>0</v>
       </c>
       <c r="T7">
         <v>0</v>
@@ -806,10 +802,10 @@
     </row>
     <row r="8" spans="1:26">
       <c r="A8">
-        <v>5.0000000000000001E-3</v>
+        <v>0</v>
       </c>
       <c r="B8">
-        <v>3.0000000000000001E-3</v>
+        <v>0</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -833,28 +829,28 @@
         <v>0</v>
       </c>
       <c r="J8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K8">
+        <v>0.3</v>
+      </c>
+      <c r="L8">
+        <v>0.2</v>
+      </c>
+      <c r="M8">
+        <v>0</v>
+      </c>
+      <c r="N8">
         <v>0.1</v>
       </c>
-      <c r="L8">
-        <v>0</v>
-      </c>
-      <c r="M8">
-        <v>0</v>
-      </c>
-      <c r="N8">
-        <v>0.5</v>
-      </c>
       <c r="O8">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
       <c r="P8">
         <v>0</v>
       </c>
       <c r="Q8">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="R8">
         <v>0</v>
@@ -916,25 +912,25 @@
         <v>0</v>
       </c>
       <c r="K9">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="L9">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="M9">
         <v>0</v>
       </c>
       <c r="N9">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="O9">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="P9">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="Q9">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="R9">
         <v>0</v>
@@ -966,10 +962,10 @@
     </row>
     <row r="10" spans="1:26">
       <c r="A10">
-        <v>0</v>
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="B10">
-        <v>0</v>
+        <v>3.0000000000000001E-3</v>
       </c>
       <c r="C10">
         <v>0</v>
@@ -990,28 +986,28 @@
         <v>0</v>
       </c>
       <c r="I10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J10">
         <v>0</v>
       </c>
       <c r="K10">
+        <v>0</v>
+      </c>
+      <c r="L10">
+        <v>0.4</v>
+      </c>
+      <c r="M10">
+        <v>0</v>
+      </c>
+      <c r="N10">
+        <v>0</v>
+      </c>
+      <c r="O10">
+        <v>0</v>
+      </c>
+      <c r="P10">
         <v>0.2</v>
-      </c>
-      <c r="L10">
-        <v>0</v>
-      </c>
-      <c r="M10">
-        <v>0</v>
-      </c>
-      <c r="N10">
-        <v>0</v>
-      </c>
-      <c r="O10">
-        <v>0</v>
-      </c>
-      <c r="P10">
-        <v>0</v>
       </c>
       <c r="Q10">
         <v>0</v>
@@ -1070,13 +1066,13 @@
         <v>0</v>
       </c>
       <c r="I11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J11">
         <v>0</v>
       </c>
       <c r="K11">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="L11">
         <v>0</v>
@@ -1103,7 +1099,7 @@
         <v>0</v>
       </c>
       <c r="T11">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="U11">
         <v>0</v>
@@ -1156,7 +1152,7 @@
         <v>0</v>
       </c>
       <c r="K12">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="L12">
         <v>0</v>
@@ -1183,7 +1179,7 @@
         <v>0</v>
       </c>
       <c r="T12">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="U12">
         <v>0</v>
@@ -1221,13 +1217,13 @@
         <v>0</v>
       </c>
       <c r="F13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I13">
         <v>0</v>
@@ -1236,22 +1232,22 @@
         <v>0</v>
       </c>
       <c r="K13">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="L13">
         <v>0</v>
       </c>
       <c r="M13">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="N13">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="O13">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="P13">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="Q13">
         <v>0</v>
@@ -1301,13 +1297,13 @@
         <v>0</v>
       </c>
       <c r="F14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I14">
         <v>0</v>
@@ -1316,22 +1312,22 @@
         <v>0</v>
       </c>
       <c r="K14">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="L14">
         <v>0</v>
       </c>
       <c r="M14">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="N14">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="O14">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="P14">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="Q14">
         <v>0</v>
@@ -1355,13 +1351,13 @@
         <v>0</v>
       </c>
       <c r="X14">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="Y14">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="Z14">
-        <v>0.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:26">
@@ -1432,16 +1428,16 @@
         <v>0</v>
       </c>
       <c r="W15">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X15">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="Y15">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="Z15">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="16" spans="1:26">
@@ -1509,10 +1505,10 @@
         <v>0</v>
       </c>
       <c r="V16">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="W16">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X16">
         <v>0</v>
@@ -1749,7 +1745,7 @@
         <v>0</v>
       </c>
       <c r="V19">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="W19">
         <v>0</v>
@@ -5446,81 +5442,161 @@
     </row>
     <row r="66" spans="1:26">
       <c r="A66">
+        <v>0</v>
+      </c>
+      <c r="B66">
+        <v>0</v>
+      </c>
+      <c r="C66">
+        <v>0</v>
+      </c>
+      <c r="D66">
+        <v>0</v>
+      </c>
+      <c r="E66">
+        <v>0</v>
+      </c>
+      <c r="F66">
+        <v>0</v>
+      </c>
+      <c r="G66">
+        <v>0</v>
+      </c>
+      <c r="H66">
+        <v>0</v>
+      </c>
+      <c r="I66">
+        <v>0</v>
+      </c>
+      <c r="J66">
+        <v>0</v>
+      </c>
+      <c r="K66">
+        <v>0</v>
+      </c>
+      <c r="L66">
+        <v>0</v>
+      </c>
+      <c r="M66">
+        <v>0</v>
+      </c>
+      <c r="N66">
+        <v>0</v>
+      </c>
+      <c r="O66">
+        <v>0</v>
+      </c>
+      <c r="P66">
+        <v>0</v>
+      </c>
+      <c r="Q66">
+        <v>0</v>
+      </c>
+      <c r="R66">
+        <v>0</v>
+      </c>
+      <c r="S66">
+        <v>0</v>
+      </c>
+      <c r="T66">
+        <v>0</v>
+      </c>
+      <c r="U66">
+        <v>0</v>
+      </c>
+      <c r="V66">
+        <v>0</v>
+      </c>
+      <c r="W66">
+        <v>0</v>
+      </c>
+      <c r="X66">
+        <v>0</v>
+      </c>
+      <c r="Y66">
+        <v>0</v>
+      </c>
+      <c r="Z66">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" spans="1:26">
+      <c r="A67">
         <v>0.99</v>
       </c>
-      <c r="B66">
+      <c r="B67">
         <v>0.99399999999999999</v>
       </c>
-      <c r="C66">
+      <c r="C67">
         <v>1</v>
       </c>
-      <c r="D66">
+      <c r="D67">
         <v>1</v>
       </c>
-      <c r="E66">
+      <c r="E67">
         <v>1</v>
       </c>
-      <c r="F66">
-        <v>0</v>
-      </c>
-      <c r="G66">
-        <v>0</v>
-      </c>
-      <c r="H66">
-        <v>0</v>
-      </c>
-      <c r="I66">
-        <v>0</v>
-      </c>
-      <c r="J66">
-        <v>0</v>
-      </c>
-      <c r="K66">
+      <c r="F67">
+        <v>0</v>
+      </c>
+      <c r="G67">
+        <v>0</v>
+      </c>
+      <c r="H67">
+        <v>0</v>
+      </c>
+      <c r="I67">
+        <v>0</v>
+      </c>
+      <c r="J67">
+        <v>0</v>
+      </c>
+      <c r="K67">
         <v>0.1</v>
       </c>
-      <c r="L66">
+      <c r="L67">
         <v>0.2</v>
       </c>
-      <c r="M66">
+      <c r="M67">
         <v>0.30000000000000004</v>
       </c>
-      <c r="N66">
+      <c r="N67">
         <v>0.30000000000000004</v>
       </c>
-      <c r="O66">
+      <c r="O67">
         <v>0.30000000000000004</v>
       </c>
-      <c r="P66">
+      <c r="P67">
         <v>0.5</v>
       </c>
-      <c r="Q66">
+      <c r="Q67">
         <v>0.5</v>
       </c>
-      <c r="R66">
-        <v>0</v>
-      </c>
-      <c r="S66">
-        <v>0</v>
-      </c>
-      <c r="T66">
+      <c r="R67">
+        <v>0</v>
+      </c>
+      <c r="S67">
+        <v>0</v>
+      </c>
+      <c r="T67">
         <v>0.9</v>
       </c>
-      <c r="U66">
+      <c r="U67">
         <v>1</v>
       </c>
-      <c r="V66">
+      <c r="V67">
         <v>0.7</v>
       </c>
-      <c r="W66">
-        <v>0</v>
-      </c>
-      <c r="X66">
+      <c r="W67">
+        <v>0</v>
+      </c>
+      <c r="X67">
         <v>0.9</v>
       </c>
-      <c r="Y66">
+      <c r="Y67">
         <v>0.9</v>
       </c>
-      <c r="Z66">
+      <c r="Z67">
         <v>0.9</v>
       </c>
     </row>

</xml_diff>